<commit_message>
Reorganize Python course materials
</commit_message>
<xml_diff>
--- a/AgenticAI/ROADMAP-AgenticAI.xlsx
+++ b/AgenticAI/ROADMAP-AgenticAI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hi\Desktop\projects\python_projects\tutorial\tut_youtube\AgenticAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2F7678-A711-4802-B155-F73F379662E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91640AC9-1789-4FD7-83DD-F6C5E3673A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1185" yWindow="2055" windowWidth="27615" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3015" yWindow="2460" windowWidth="25455" windowHeight="12870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="112">
   <si>
     <t>Category</t>
   </si>
@@ -349,6 +349,18 @@
   </si>
   <si>
     <t>email agent</t>
+  </si>
+  <si>
+    <t>Agentic RAG</t>
+  </si>
+  <si>
+    <t>Definition and difference fro traditional RAG</t>
+  </si>
+  <si>
+    <t>RAG</t>
+  </si>
+  <si>
+    <t>done</t>
   </si>
 </sst>
 </file>
@@ -690,7 +702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.42578125" style="3" customWidth="1"/>
@@ -1002,26 +1014,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D23" s="4"/>
-      <c r="E23" s="3"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" s="3">
-        <v>30</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>75</v>
-      </c>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D24" s="4"/>
+      <c r="E24" s="3"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
@@ -1031,13 +1026,13 @@
         <v>30</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D26" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1045,13 +1040,16 @@
         <v>91</v>
       </c>
       <c r="B27" s="3">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>77</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1062,10 +1060,10 @@
         <v>25</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D28" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1073,73 +1071,60 @@
         <v>91</v>
       </c>
       <c r="B29" s="3">
+        <v>25</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B30" s="3">
         <v>20</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C30" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D30" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B31" s="3">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
       <c r="D31" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="E31" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C32" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B32" s="3">
-        <v>35</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" t="s">
-        <v>45</v>
-      </c>
-    </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B33" s="3">
-        <v>40</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D33" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B34" s="3">
-        <v>35</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D34" t="s">
-        <v>49</v>
-      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="3"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
@@ -1149,191 +1134,250 @@
         <v>30</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D35" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
+      </c>
+      <c r="B36" s="3">
+        <v>35</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="D36" t="s">
-        <v>103</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
+      </c>
+      <c r="B37" s="3">
+        <v>40</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>76</v>
+        <v>46</v>
+      </c>
+      <c r="D37" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E38" s="3"/>
+      <c r="A38" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B38" s="3">
+        <v>35</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D38" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="3">
+        <v>30</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" t="s">
+        <v>81</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B40" s="3">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="D40" t="s">
-        <v>53</v>
+        <v>103</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="3"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="3">
-        <v>25</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D41" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B42" s="3">
-        <v>30</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D42" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B43" s="3">
-        <v>25</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D43" t="s">
-        <v>59</v>
+      <c r="B44" s="3">
+        <v>30</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D44" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B45" s="3">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D45" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B46" s="3">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D46" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B47" s="3">
         <v>25</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D47" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B49" s="3">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D49" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B50" s="3">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D50" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B51" s="3">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D51" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53" s="3">
+        <v>60</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D53" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="3">
+        <v>30</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D54" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" s="3">
+        <v>20</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D55" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C57" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D57" t="s">
         <v>100</v>
       </c>
     </row>

</xml_diff>